<commit_message>
lab name update and stats link in home page
</commit_message>
<xml_diff>
--- a/excels/LabDetails.xlsx
+++ b/excels/LabDetails.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\code\nitw\NITW-Transportation-Division\excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5954A45-C7A0-4BF0-B53C-534EC3FE67A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3910C0BA-74A8-49C8-BE0F-4EB13658EE7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="111">
   <si>
     <t>CUBE 5</t>
   </si>
@@ -358,6 +358,21 @@
   </si>
   <si>
     <t>Gyrocomp</t>
+  </si>
+  <si>
+    <t>Lab</t>
+  </si>
+  <si>
+    <t>Transportation Software</t>
+  </si>
+  <si>
+    <t>Pavement Material &amp; Evaluation</t>
+  </si>
+  <si>
+    <t>Advanced Pavement Materials Testing</t>
+  </si>
+  <si>
+    <t>Transportation Engineering</t>
   </si>
 </sst>
 </file>
@@ -687,7 +702,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D19"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="37.85546875" customWidth="1"/>
@@ -696,7 +711,7 @@
     <col min="4" max="4" width="48.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>16</v>
       </c>
@@ -709,8 +724,11 @@
       <c r="D1" s="1" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="E1" s="1" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>17</v>
       </c>
@@ -723,8 +741,11 @@
       <c r="D2" s="2" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+      <c r="E2" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="45" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
         <v>1</v>
       </c>
@@ -735,7 +756,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" ht="45" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
         <v>2</v>
       </c>
@@ -746,7 +767,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="60" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" ht="60" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
         <v>3</v>
       </c>
@@ -757,7 +778,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" ht="45" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
         <v>4</v>
       </c>
@@ -768,7 +789,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" ht="45" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
         <v>5</v>
       </c>
@@ -776,7 +797,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
         <v>6</v>
       </c>
@@ -784,45 +805,45 @@
         <v>73</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
         <v>7</v>
       </c>
       <c r="D9" s="2"/>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
         <v>8</v>
       </c>
       <c r="D10" s="2"/>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
         <v>9</v>
       </c>
       <c r="D11" s="2"/>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B14" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B15" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B16" t="s">
         <v>13</v>
       </c>
@@ -845,7 +866,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:D29"/>
+  <dimension ref="A1:E29"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="19" customWidth="1"/>
@@ -853,7 +874,7 @@
     <col min="4" max="4" width="73.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>16</v>
       </c>
@@ -866,8 +887,11 @@
       <c r="D1" s="1" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1" s="1" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>20</v>
       </c>
@@ -877,8 +901,11 @@
       <c r="D2" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E2" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C3" t="s">
         <v>22</v>
       </c>
@@ -886,7 +913,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C4" t="s">
         <v>23</v>
       </c>
@@ -894,7 +921,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C5" t="s">
         <v>24</v>
       </c>
@@ -902,7 +929,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C6" t="s">
         <v>25</v>
       </c>
@@ -910,7 +937,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C7" t="s">
         <v>26</v>
       </c>
@@ -918,7 +945,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C8" t="s">
         <v>27</v>
       </c>
@@ -926,7 +953,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C9" t="s">
         <v>28</v>
       </c>
@@ -934,7 +961,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C10" t="s">
         <v>29</v>
       </c>
@@ -942,7 +969,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C11" t="s">
         <v>30</v>
       </c>
@@ -950,7 +977,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C12" t="s">
         <v>31</v>
       </c>
@@ -958,7 +985,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C13" t="s">
         <v>32</v>
       </c>
@@ -966,7 +993,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C14" t="s">
         <v>33</v>
       </c>
@@ -974,7 +1001,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C15" t="s">
         <v>34</v>
       </c>
@@ -982,7 +1009,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C16" t="s">
         <v>35</v>
       </c>
@@ -1071,7 +1098,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1AA06181-9D79-4C6D-B340-48ADABA23ABA}">
-  <dimension ref="A1:D20"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.42578125" bestFit="1" customWidth="1"/>
@@ -1080,7 +1107,7 @@
     <col min="4" max="4" width="118.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>16</v>
       </c>
@@ -1093,8 +1120,11 @@
       <c r="D1" s="1" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1" s="1" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
         <v>86</v>
       </c>
@@ -1104,8 +1134,11 @@
       <c r="D2" t="s">
         <v>91</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E2" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
         <v>87</v>
       </c>
@@ -1116,7 +1149,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
         <v>88</v>
       </c>
@@ -1127,7 +1160,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
         <v>89</v>
       </c>
@@ -1138,7 +1171,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
         <v>90</v>
       </c>
@@ -1149,52 +1182,52 @@
         <v>52</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="D7" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="D8" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="D9" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="D10" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="D11" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="D12" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="D13" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="D14" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="D15" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="D16" t="s">
         <v>62</v>
       </c>
@@ -1226,7 +1259,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BD3B26B7-960D-4148-BDF8-5BFAAD40DC3E}">
-  <dimension ref="A1:D19"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.42578125" bestFit="1" customWidth="1"/>
@@ -1235,7 +1268,7 @@
     <col min="4" max="4" width="118.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>16</v>
       </c>
@@ -1248,8 +1281,11 @@
       <c r="D1" s="1" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1" s="1" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
         <v>105</v>
       </c>
@@ -1259,8 +1295,11 @@
       <c r="D2" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E2" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C3" t="s">
         <v>93</v>
       </c>
@@ -1268,7 +1307,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C4" t="s">
         <v>94</v>
       </c>
@@ -1276,7 +1315,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C5" t="s">
         <v>95</v>
       </c>
@@ -1284,7 +1323,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C6" t="s">
         <v>96</v>
       </c>
@@ -1292,7 +1331,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C7" t="s">
         <v>97</v>
       </c>
@@ -1300,7 +1339,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C8" t="s">
         <v>98</v>
       </c>
@@ -1308,7 +1347,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C9" t="s">
         <v>99</v>
       </c>
@@ -1316,7 +1355,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C10" t="s">
         <v>100</v>
       </c>
@@ -1324,7 +1363,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C11" t="s">
         <v>101</v>
       </c>
@@ -1332,7 +1371,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C12" t="s">
         <v>102</v>
       </c>
@@ -1340,7 +1379,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C13" t="s">
         <v>103</v>
       </c>
@@ -1348,7 +1387,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C14" t="s">
         <v>36</v>
       </c>
@@ -1356,7 +1395,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C15" t="s">
         <v>104</v>
       </c>
@@ -1364,7 +1403,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="D16" t="s">
         <v>63</v>
       </c>

</xml_diff>